<commit_message>
순위 수집 2026-07-31 19:04 KST
</commit_message>
<xml_diff>
--- a/docs/report.xlsx
+++ b/docs/report.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="순위추이" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시간대별" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변동성" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="순위이력" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="순위추이" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="시간대별" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="변동성" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="순위이력" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,11 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF006300"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -76,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -84,6 +89,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -158,6 +164,734 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>중고차팔기 순위 추이</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!B5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$B$6:$B$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!C5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$C$6:$C$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$D$6:$D$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$E$6:$E$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>조회시각</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>노출순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>내차팔기 순위 추이</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!B22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$B$23:$B$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!C22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$C$23:$C$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!D22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$D$23:$D$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!E22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$E$23:$E$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>조회시각</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>노출순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>내차시세조회 순위 추이</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!B39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$B$40:$B$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!C39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$C$40:$C$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!D39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$D$40:$D$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!E39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$E$40:$E$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>조회시각</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>노출순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,7 +1205,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준 업체 엔카 · 최근 720시간 · 생성 2026-07-31 19:02 · 모바일 파워링크 기준(1페이지 15개)</t>
+          <t>기준 업체 엔카 · 최근 720시간 · 생성 2026-07-31 19:04 · 모바일 파워링크 기준(1페이지 15개)</t>
         </is>
       </c>
     </row>
@@ -506,11 +1240,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>비교할 직전 기록 없음</t>
+        <v>2</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>▲ 4.3위</t>
         </is>
       </c>
     </row>
@@ -525,7 +1259,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>비교할 직전 기록 없음</t>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -536,11 +1270,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>비교할 직전 기록 없음</t>
+        <v>3</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>▲ 3개</t>
         </is>
       </c>
     </row>
@@ -555,7 +1289,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>비교할 직전 기록 없음</t>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -603,13 +1337,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -617,11 +1351,11 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>73</v>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>44</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>▲ 5</t>
         </is>
       </c>
     </row>
@@ -632,25 +1366,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
+        <v>17</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>33</v>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>순위밖</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>56</v>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>▲ 3</t>
         </is>
       </c>
     </row>
@@ -661,13 +1395,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -675,11 +1409,11 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>35</v>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>25</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>▲ 5</t>
         </is>
       </c>
     </row>
@@ -713,7 +1447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -739,14 +1473,206 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>추이를 그리려면 같은 키워드로 2회 이상 수집되어야 합니다.</t>
-        </is>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>조회시각</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>07-31 19:02</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>07-31 19:04</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>조회시각</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07-31 19:02</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07-31 19:04</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>조회시각</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07-31 19:02</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07-31 19:04</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -777,7 +1703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>엔카 기준 — 가장 좋은 시간대 19시(평균 6.3위) · 가장 밀리는 시간대 19시(평균 6.3위)</t>
+          <t>엔카 기준 — 가장 좋은 시간대 19시(평균 4.2위) · 가장 밀리는 시간대 19시(평균 4.2위)</t>
         </is>
       </c>
     </row>
@@ -820,16 +1746,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.3</v>
+        <v>4.2</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
       <c r="D5" t="n">
-        <v>33.3</v>
+        <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -924,7 +1850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1400,6 +2326,420 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>44</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3,3,3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>44</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>27</v>
+      </c>
+      <c r="E18" t="n">
+        <v>44</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>27,27,27</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>44</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>33</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2,2,2</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>33</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>17</v>
+      </c>
+      <c r="E22" t="n">
+        <v>33</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>17,17,17</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>33</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>25</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>25</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2,2,2</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>12</v>
+      </c>
+      <c r="E26" t="n">
+        <v>25</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>12,12,12</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:04:17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>25</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
순위 수집 2026-07-31 19:05 KST
</commit_message>
<xml_diff>
--- a/docs/report.xlsx
+++ b/docs/report.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,11 +43,6 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF006300"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -81,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -89,7 +84,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -211,12 +205,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$6:$A$7</f>
+              <f>'순위추이'!$A$6:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$B$6:$B$7</f>
+              <f>'순위추이'!$B$6:$B$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -244,12 +238,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$6:$A$7</f>
+              <f>'순위추이'!$A$6:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$C$6:$C$7</f>
+              <f>'순위추이'!$C$6:$C$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -277,12 +271,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$6:$A$7</f>
+              <f>'순위추이'!$A$6:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$D$6:$D$7</f>
+              <f>'순위추이'!$D$6:$D$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -310,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$6:$A$7</f>
+              <f>'순위추이'!$A$6:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$E$6:$E$7</f>
+              <f>'순위추이'!$E$6:$E$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -430,12 +424,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$23:$A$24</f>
+              <f>'순위추이'!$A$23:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$B$23:$B$24</f>
+              <f>'순위추이'!$B$23:$B$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -463,12 +457,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$23:$A$24</f>
+              <f>'순위추이'!$A$23:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$C$23:$C$24</f>
+              <f>'순위추이'!$C$23:$C$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -496,12 +490,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$23:$A$24</f>
+              <f>'순위추이'!$A$23:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$D$23:$D$24</f>
+              <f>'순위추이'!$D$23:$D$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -529,12 +523,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$23:$A$24</f>
+              <f>'순위추이'!$A$23:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$E$23:$E$24</f>
+              <f>'순위추이'!$E$23:$E$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -649,12 +643,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$40:$A$41</f>
+              <f>'순위추이'!$A$40:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$B$40:$B$41</f>
+              <f>'순위추이'!$B$40:$B$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -682,12 +676,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$40:$A$41</f>
+              <f>'순위추이'!$A$40:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$C$40:$C$41</f>
+              <f>'순위추이'!$C$40:$C$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -715,12 +709,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$40:$A$41</f>
+              <f>'순위추이'!$A$40:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$D$40:$D$41</f>
+              <f>'순위추이'!$D$40:$D$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -748,12 +742,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'순위추이'!$A$40:$A$41</f>
+              <f>'순위추이'!$A$40:$A$42</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'순위추이'!$E$40:$E$41</f>
+              <f>'순위추이'!$E$40:$E$42</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1205,7 +1199,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준 업체 엔카 · 최근 720시간 · 생성 2026-07-31 19:04 · 모바일 파워링크 기준(1페이지 15개)</t>
+          <t>기준 업체 엔카 · 최근 720시간 · 생성 2026-07-31 19:05 · 모바일 파워링크 기준(1페이지 15개)</t>
         </is>
       </c>
     </row>
@@ -1242,9 +1236,9 @@
       <c r="B6" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>▲ 4.3위</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -1272,9 +1266,9 @@
       <c r="B8" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>▲ 3개</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -1353,9 +1347,9 @@
       <c r="F13" t="n">
         <v>44</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>▲ 5</t>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -1382,9 +1376,9 @@
       <c r="F14" t="n">
         <v>33</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>▲ 3</t>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -1411,9 +1405,9 @@
       <c r="F15" t="n">
         <v>25</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>▲ 5</t>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1538,6 +1532,22 @@
         <v>27</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07-31 19:05</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>27</v>
+      </c>
+    </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -1604,6 +1614,22 @@
         <v>17</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07-31 19:05</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>17</v>
+      </c>
+    </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
@@ -1667,6 +1693,22 @@
         <v>2</v>
       </c>
       <c r="D41" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07-31 19:05</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1703,7 +1745,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>엔카 기준 — 가장 좋은 시간대 19시(평균 4.2위) · 가장 밀리는 시간대 19시(평균 4.2위)</t>
+          <t>엔카 기준 — 가장 좋은 시간대 19시(평균 3.4위) · 가장 밀리는 시간대 19시(평균 3.4위)</t>
         </is>
       </c>
     </row>
@@ -1746,16 +1788,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.2</v>
+        <v>3.4</v>
       </c>
       <c r="C5" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>23.6</v>
       </c>
       <c r="F5" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1769,7 +1811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1833,10 +1875,219 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>표본이 3회 미만이라 아직 계산할 수 없습니다.</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="D5" t="n">
+        <v>27</v>
+      </c>
+      <c r="E5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="D6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E6" t="n">
+        <v>33</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1850,7 +2101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2740,6 +2991,420 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>44</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>3,3,3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>44</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>27</v>
+      </c>
+      <c r="E30" t="n">
+        <v>44</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>27,27,27</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>44</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>33</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2,2,2</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>33</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>17</v>
+      </c>
+      <c r="E34" t="n">
+        <v>33</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>17,17,17</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>33</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>25</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>25</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2,2,2</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>12</v>
+      </c>
+      <c r="E38" t="n">
+        <v>25</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>12,12,12</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-31 19:05:45</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>25</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
순위 수집 2026-08-16 14:29 KST
</commit_message>
<xml_diff>
--- a/docs/report.xlsx
+++ b/docs/report.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="순위추이" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시간대별" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="변동성" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="순위이력" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="순위추이" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="시간대별" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="변동성" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="순위이력" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,11 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFD03B3B"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -76,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -84,6 +89,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -158,6 +164,945 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>중고차팔기 순위 추이</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!B5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$B$6:$B$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!C5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$C$6:$C$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$D$6:$D$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$6:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$E$6:$E$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>조회시각</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>노출순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>내차팔기 순위 추이</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!B22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$B$23:$B$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!C22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$C$23:$C$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!D22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$D$23:$D$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!E22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$23:$A$24</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$E$23:$E$24</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>조회시각</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>노출순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>내차시세조회 순위 추이</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!B39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$B$40:$B$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!C39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$C$40:$C$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!D39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$D$40:$D$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'순위추이'!E39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'순위추이'!$A$40:$A$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'순위추이'!$E$40:$E$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>조회시각</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>노출순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>시간대별 평균 노출순위 (낮을수록 상위)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'시간대별'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'시간대별'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'시간대별'!$B$5:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'시간대별'!C4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'시간대별'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'시간대별'!$C$5:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'시간대별'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'시간대별'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'시간대별'!$D$5:$D$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'시간대별'!E4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'시간대별'!$A$5:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'시간대별'!$E$5:$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>시간</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>평균 순위</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,7 +1416,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준 업체 엔카 · 최근 720시간 · 생성 2026-08-03 14:42 · 모바일 파워링크 기준(1페이지 15개)</t>
+          <t>기준 업체 엔카 · 최근 720시간 · 생성 2026-08-16 14:29 · 모바일 파워링크 기준(1페이지 15개)</t>
         </is>
       </c>
     </row>
@@ -505,8 +1450,10 @@
           <t>평균 순위</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>6.3</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -521,11 +1468,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>비교할 직전 기록 없음</t>
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>▼ 3개</t>
         </is>
       </c>
     </row>
@@ -540,7 +1487,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>비교할 직전 기록 없음</t>
+          <t>변화 없음</t>
         </is>
       </c>
     </row>
@@ -551,11 +1498,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>비교할 직전 기록 없음</t>
+        <v>3</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>▲ 3개</t>
         </is>
       </c>
     </row>
@@ -602,14 +1549,18 @@
           <t>중고차팔기</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>8</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
       </c>
       <c r="C13" t="n">
         <v>1</v>
       </c>
-      <c r="D13" t="n">
-        <v>45</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -617,7 +1568,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -631,14 +1582,18 @@
           <t>내차팔기</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>5</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="n">
-        <v>33</v>
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -646,7 +1601,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -660,14 +1615,18 @@
           <t>내차시세조회</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>6</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
-      </c>
-      <c r="D15" t="n">
-        <v>22</v>
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -675,7 +1634,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -713,7 +1672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -739,14 +1698,188 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>추이를 그리려면 같은 키워드로 2회 이상 수집되어야 합니다.</t>
-        </is>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>조회시각</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>07-31 19:02</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08-16 14:29</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>조회시각</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07-31 19:02</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08-16 14:29</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>조회시각</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07-31 19:02</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08-16 14:29</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -756,7 +1889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -816,24 +1949,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>19시</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>6.3</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C6" t="n">
         <v>3.3</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D6" t="n">
         <v>33.3</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F6" t="n">
         <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -924,7 +2071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1400,6 +2547,432 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>43</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>43</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1,1,1</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>43</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>중고차팔기</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>43</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>37</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>37</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2,2,2</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>37</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>내차팔기</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>37</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>엔카</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>27</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>헤이딜러</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>27</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2,2,2</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>K다이렉트카</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>27</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-16 14:29:38</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>내차시세조회</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>현대글로비스오토벨</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>순위밖</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>27</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>-,-,-</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>수동</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>